<commit_message>
PAUSED (task172): stage 4 round 4, the ask layer re-sited off the scored reader's path, call side byte-identical
The round 4 reader kept 14 of 14 ask figures; each device now sits on a join that path does not make, with every
ask, rounding, pin and golden figure unchanged: the first (c)(9) cards' approvals only in the green-card tracker, a
spouse employed at Sallowmere under her employee ID and her spouse ID (one card number), an employee moved between
Sallowmere entities under two HR IDs (one enrollment), the applicant's own refiling as a case of its own beside the
team's case closed not refiled, and applicants' forwarded rejections of their own other filings dated outside the
renewal's packets. The cracker (that reader's path) keeps 0 of 20 ask cells; every call computation is identical to
the round 3 commit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task172/golden/q1_2027_renewal_quote.xlsx
+++ b/task172/golden/q1_2027_renewal_quote.xlsx
@@ -133,7 +133,7 @@
     <t>July to September 2027</t>
   </si>
   <si>
-    <t>Each current person's work permit (GM-07 1.3 and 1.4): the card USCIS approved most recently, from HR's roster, counsel's approval notices, the case register and the green-card tracker, in the category of the approval. A spouse is counted once, whether Global Mobility's records or Benefits' ID carries her card, and belongs to the household the register, the tracker, the roster's onboarding entry or Benefits names.</t>
+    <t>Each current person's work permit (GM-07 1.3 and 1.4): the card USCIS approved most recently, from HR's roster, counsel's approval notices, the case register and the green-card tracker, in the category of the approval. Each person is counted once under all her IDs: an employee under every ID HR's program roster gives him (one benefits enrollment), a spouse whether Global Mobility's records, Benefits' ID or her own employee ID carries her card (one card number); a spouse belongs to the household the register, the tracker, the roster's onboarding entry or Benefits names.</t>
   </si>
   <si>
     <t>Most rejected renewal packets were filed again within 30 days</t>
@@ -166,7 +166,7 @@
     <t>October 2025 to September 2026</t>
   </si>
   <si>
-    <t>Rejection notices counsel logged and those applicants forwarded to Global Mobility, one per case and notice date. Filed again within 30 days means USCIS received the renewal again no later than the 30th day after the notice's date (GM-07 2.3 and 2.4), whoever filed it.</t>
+    <t>Rejection notices counsel logged and those applicants forwarded to Global Mobility, one per renewal and notice date, dated after the renewal's first packet left the mailroom and before USCIS had the renewal (the others are rejections of applicants' own other filings). Filed again within 30 days means USCIS received the renewal again no later than the 30th day after the notice's date (GM-07 2.3 and 2.4), whoever filed it and whichever case the register holds it under.</t>
   </si>
 </sst>
 </file>
@@ -789,7 +789,7 @@
         <v>1622</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ht="84" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>35</v>
       </c>
@@ -888,7 +888,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="40" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="92" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>46</v>
       </c>

</xml_diff>